<commit_message>
New Architecture with better Accuracy
</commit_message>
<xml_diff>
--- a/AutoEIT_Developer_Matrix_Full_Data.xlsx
+++ b/AutoEIT_Developer_Matrix_Full_Data.xlsx
@@ -770,7 +770,7 @@
         <v>0.375</v>
       </c>
       <c r="O6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -823,7 +823,7 @@
         <v>0.1666666666666667</v>
       </c>
       <c r="O7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -876,7 +876,7 @@
         <v>0.125</v>
       </c>
       <c r="O8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -982,7 +982,7 @@
         <v>0.1428571428571428</v>
       </c>
       <c r="O10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1088,7 +1088,7 @@
         <v>0.2222222222222222</v>
       </c>
       <c r="O12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1194,7 +1194,7 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="O14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1406,7 +1406,7 @@
         <v>0.4444444444444444</v>
       </c>
       <c r="O18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -1459,7 +1459,7 @@
         <v>0.1428571428571428</v>
       </c>
       <c r="O19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1565,7 +1565,7 @@
         <v>0.1818181818181818</v>
       </c>
       <c r="O21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1618,7 +1618,7 @@
         <v>0.2</v>
       </c>
       <c r="O22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -1830,7 +1830,7 @@
         <v>0.2</v>
       </c>
       <c r="O26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -2345,7 +2345,7 @@
         <v>0.2</v>
       </c>
       <c r="O4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -2610,7 +2610,7 @@
         <v>0.1428571428571428</v>
       </c>
       <c r="O9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -2663,7 +2663,7 @@
         <v>0.2857142857142857</v>
       </c>
       <c r="O10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -2716,7 +2716,7 @@
         <v>0.1428571428571428</v>
       </c>
       <c r="O11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -2928,7 +2928,7 @@
         <v>0.2857142857142857</v>
       </c>
       <c r="O15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -3246,7 +3246,7 @@
         <v>0.09090909090909091</v>
       </c>
       <c r="O21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -3511,7 +3511,7 @@
         <v>0.2</v>
       </c>
       <c r="O26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -3617,7 +3617,7 @@
         <v>0.2727272727272727</v>
       </c>
       <c r="O28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -4026,7 +4026,7 @@
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -4132,7 +4132,7 @@
         <v>0.25</v>
       </c>
       <c r="O6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -4291,7 +4291,7 @@
         <v>0.1428571428571428</v>
       </c>
       <c r="O9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -4397,7 +4397,7 @@
         <v>0.2857142857142857</v>
       </c>
       <c r="O11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -4450,7 +4450,7 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="O12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -4503,7 +4503,7 @@
         <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -4556,7 +4556,7 @@
         <v>0.4444444444444444</v>
       </c>
       <c r="O14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -4662,7 +4662,7 @@
         <v>0.125</v>
       </c>
       <c r="O16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -4927,7 +4927,7 @@
         <v>0.1818181818181818</v>
       </c>
       <c r="O21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -4980,7 +4980,7 @@
         <v>0.2</v>
       </c>
       <c r="O22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -5139,7 +5139,7 @@
         <v>0.375</v>
       </c>
       <c r="O25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -5192,7 +5192,7 @@
         <v>0.6</v>
       </c>
       <c r="O26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -5245,7 +5245,7 @@
         <v>0.3333333333333333</v>
       </c>
       <c r="O27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -5298,7 +5298,7 @@
         <v>0.09090909090909091</v>
       </c>
       <c r="O28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -5457,7 +5457,7 @@
         <v>0.1</v>
       </c>
       <c r="O31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -5707,7 +5707,7 @@
         <v>0.4</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -5760,7 +5760,7 @@
         <v>0.2</v>
       </c>
       <c r="O5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -5866,7 +5866,7 @@
         <v>0.3333333333333333</v>
       </c>
       <c r="O7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -5919,7 +5919,7 @@
         <v>0.125</v>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -6078,7 +6078,7 @@
         <v>0.1428571428571428</v>
       </c>
       <c r="O11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -6131,7 +6131,7 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="O12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -6184,7 +6184,7 @@
         <v>0.25</v>
       </c>
       <c r="O13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -6290,7 +6290,7 @@
         <v>0.1428571428571428</v>
       </c>
       <c r="O15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -6502,7 +6502,7 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="O19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -6608,7 +6608,7 @@
         <v>0.09090909090909091</v>
       </c>
       <c r="O21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -6820,7 +6820,7 @@
         <v>0.375</v>
       </c>
       <c r="O25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -7085,7 +7085,7 @@
         <v>0</v>
       </c>
       <c r="O30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">

</xml_diff>